<commit_message>
Added T-Nuts to BOM
</commit_message>
<xml_diff>
--- a/Fila_Feeder_BOM.xlsx
+++ b/Fila_Feeder_BOM.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce874e8f9ea78aa2/Documents/3D Printing/TORBJORN BUILD FILES/Feeder Extruder/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_7852788D1C4905F7405CEB79A81B16403AB38ED2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A47E757-05D9-4AB2-B2DF-D8504E9F53DA}"/>
+  <bookViews>
+    <workbookView xWindow="-15660" yWindow="1725" windowWidth="18570" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>Bill of Materials</t>
   </si>
@@ -149,52 +158,78 @@
   </si>
   <si>
     <t>https://a.co/d/0a5YDpLx</t>
+  </si>
+  <si>
+    <t>M3 T-Nut</t>
+  </si>
+  <si>
+    <t>https://a.co/d/071vCX4D</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
-    <font>
-      <sz val="10.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="10">
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF212529"/>
       <name val="-apple-system"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF212529"/>
       <name val="-apple-system"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="-apple-system"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -202,7 +237,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -223,72 +258,102 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
-    <border/>
+  <borders count="4">
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FFDEE2E6"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF454D55"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -478,29 +543,32 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="34.25"/>
-    <col customWidth="1" min="4" max="4" width="23.63"/>
-    <col customWidth="1" min="5" max="5" width="38.5"/>
+    <col min="2" max="2" width="34.28515625" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="38.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -517,258 +585,270 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="7" t="s">
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7">
-        <v>9.0</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="C4" s="6">
+        <v>9</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="7" t="s">
+    <row r="5" spans="1:5">
+      <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="C5" s="6">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="7" t="s">
+    <row r="6" spans="1:5">
+      <c r="B6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="C6" s="6">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="7" t="s">
+    <row r="7" spans="1:5">
+      <c r="B7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="6">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="7" t="s">
+    <row r="8" spans="1:5" thickBot="1">
+      <c r="B8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="7">
-        <v>7.0</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="C8" s="6">
+        <v>7</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="7" t="s">
+    <row r="9" spans="1:5" ht="13.5" thickBot="1">
+      <c r="B9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="11">
+        <v>3</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="12.75">
+      <c r="B10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="7">
-        <v>2.0</v>
-      </c>
-      <c r="D9" s="8" t="s">
+      <c r="C10" s="6">
+        <v>2</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="s">
+    <row r="11" spans="1:5">
+      <c r="A11" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="B12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="C12" s="6">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="s">
+    <row r="13" spans="1:5">
+      <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="B14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D13" s="8" t="s">
+      <c r="C14" s="6">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="7" t="s">
+    <row r="15" spans="1:5">
+      <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D14" s="8" t="s">
+      <c r="C15" s="6">
+        <v>1</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E15" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="7" t="s">
+    <row r="16" spans="1:5">
+      <c r="B16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D15" s="8" t="s">
+      <c r="C16" s="6">
+        <v>1</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="7" t="s">
+    <row r="17" spans="1:5">
+      <c r="B17" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D16" s="8" t="s">
+      <c r="C17" s="6">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E17" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="s">
+    <row r="18" spans="1:5">
+      <c r="A18" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="B19" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="7">
-        <v>2.0</v>
-      </c>
-      <c r="D18" s="10" t="s">
+      <c r="C19" s="6">
+        <v>2</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="7" t="s">
+    <row r="20" spans="1:5">
+      <c r="B20" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="7">
-        <v>2.0</v>
-      </c>
-      <c r="D19" s="10" t="s">
+      <c r="C20" s="6">
+        <v>2</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="7" t="s">
+    <row r="21" spans="1:5">
+      <c r="B21" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="C21" s="6">
+        <v>1</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="7" t="s">
+    <row r="22" spans="1:5">
+      <c r="B22" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="C22" s="6">
+        <v>1</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="7" t="s">
+    <row r="23" spans="1:5">
+      <c r="B23" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="C23" s="6">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="7" t="s">
+    <row r="24" spans="1:5">
+      <c r="B24" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D23" s="8" t="s">
+      <c r="C24" s="6">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>45</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="D4"/>
-    <hyperlink r:id="rId2" ref="D5"/>
-    <hyperlink r:id="rId3" ref="D6"/>
-    <hyperlink r:id="rId4" ref="D7"/>
-    <hyperlink r:id="rId5" ref="D8"/>
-    <hyperlink r:id="rId6" ref="D9"/>
-    <hyperlink r:id="rId7" ref="D11"/>
-    <hyperlink r:id="rId8" ref="D13"/>
-    <hyperlink r:id="rId9" ref="D14"/>
-    <hyperlink r:id="rId10" ref="D15"/>
-    <hyperlink r:id="rId11" ref="D16"/>
-    <hyperlink r:id="rId12" ref="D18"/>
-    <hyperlink r:id="rId13" ref="D19"/>
-    <hyperlink r:id="rId14" ref="D20"/>
-    <hyperlink r:id="rId15" ref="D21"/>
-    <hyperlink r:id="rId16" ref="D22"/>
-    <hyperlink r:id="rId17" ref="D23"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D12" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D14" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D16" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D19" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D20" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D21" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D22" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="D23" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D24" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D9" r:id="rId18" xr:uid="{329EB4BB-C6FA-4490-B467-6B2FFEE10BB2}"/>
   </hyperlinks>
-  <drawing r:id="rId18"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>